<commit_message>
Fix live Excel parsing logic for Marketing, ISC & Procurement, and Strategic KPIs
</commit_message>
<xml_diff>
--- a/data/Masterfile_DMB_Dashboard.xlsx
+++ b/data/Masterfile_DMB_Dashboard.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="1" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="MPR Masterfile" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="DMB Masterfile" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MPR Masterfile" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DMB Masterfile" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -1708,6 +1708,9 @@
       <c r="R9" t="n">
         <v>1</v>
       </c>
+      <c r="S9" t="n">
+        <v>1</v>
+      </c>
       <c r="W9" t="inlineStr">
         <is>
           <t>Whole Number</t>
@@ -4957,7 +4960,11 @@
           <t>QTR</t>
         </is>
       </c>
-      <c r="S51" s="50" t="n"/>
+      <c r="S51" s="50" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
       <c r="T51" s="50" t="n"/>
       <c r="U51" s="50" t="n"/>
       <c r="V51" s="50" t="n"/>
@@ -5042,7 +5049,7 @@
         </is>
       </c>
       <c r="P52" s="39" t="n">
-        <v>0.121</v>
+        <v>0.12</v>
       </c>
       <c r="Q52" s="8" t="inlineStr">
         <is>
@@ -5050,6 +5057,11 @@
         </is>
       </c>
       <c r="R52" s="8" t="inlineStr">
+        <is>
+          <t>QTR</t>
+        </is>
+      </c>
+      <c r="S52" t="inlineStr">
         <is>
           <t>QTR</t>
         </is>
@@ -5473,7 +5485,11 @@
         </is>
       </c>
       <c r="R59" s="12" t="n"/>
-      <c r="S59" s="12" t="n"/>
+      <c r="S59" s="12" t="inlineStr">
+        <is>
+          <t>HY</t>
+        </is>
+      </c>
       <c r="T59" s="12" t="n"/>
       <c r="U59" s="12" t="n"/>
       <c r="V59" s="12" t="n"/>
@@ -9053,17 +9069,17 @@
       </c>
       <c r="R47" s="4" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="S47" s="4" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="T47" s="4" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="U47" t="inlineStr">
@@ -9147,17 +9163,17 @@
       </c>
       <c r="R48" s="4" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="S48" s="4" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="T48" s="4" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="U48" t="inlineStr">
@@ -11281,26 +11297,6 @@
       <c r="J74" t="n">
         <v>7</v>
       </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N74" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="O74" t="n">
         <v>0</v>
       </c>
@@ -11805,10 +11801,8 @@
       <c r="P80" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="Q80" s="12" t="inlineStr">
-        <is>
-          <t>90%%</t>
-        </is>
+      <c r="Q80" s="12" t="n">
+        <v>0.9</v>
       </c>
       <c r="R80" s="12" t="n"/>
       <c r="S80" s="12" t="n"/>
@@ -11949,36 +11943,12 @@
           <t>Actual</t>
         </is>
       </c>
-      <c r="I82" s="34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J82" s="34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K82" s="34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L82" s="34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M82" s="34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N82" s="34" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="I82" s="34" t="n"/>
+      <c r="J82" s="34" t="n"/>
+      <c r="K82" s="34" t="n"/>
+      <c r="L82" s="34" t="n"/>
+      <c r="M82" s="34" t="n"/>
+      <c r="N82" s="34" t="n"/>
       <c r="O82" s="20" t="n">
         <v>1</v>
       </c>
@@ -14328,10 +14298,8 @@
       <c r="P112" s="2" t="n">
         <v>0.345</v>
       </c>
-      <c r="Q112" s="3" t="inlineStr">
-        <is>
-          <t>35.2%</t>
-        </is>
+      <c r="Q112" s="3" t="n">
+        <v>0.352</v>
       </c>
       <c r="R112" s="2" t="n"/>
       <c r="S112" s="2" t="n"/>

</xml_diff>